<commit_message>
test(mercado): planilha de amostra no leiaute conferido na planilha real
</commit_message>
<xml_diff>
--- a/packages/mercado/testes/fixtures/revendas_lpc_amostra.xlsx
+++ b/packages/mercado/testes/fixtures/revendas_lpc_amostra.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,340 +431,157 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LEVANTAMENTO DE PREÇOS DE COMBUSTÍVEIS - PREÇOS PRATICADOS POR REVENDA</t>
+          <t>SUPERINTENDÊNCIA DE DEFESA DA CONCORRÊNCIA</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PERÍODO: 28/09/2026 A 03/10/2026</t>
+          <t>SISTEMA DE LEVANTAMENTO DE PREÇOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>INTERVALO DE TEMPO: SEMANAL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CNPJ</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>RAZÃO</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>FANTASIA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>ENDEREÇO</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>NÚMERO</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>COMPLEMENTO</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>BAIRRO</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>CEP</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>MUNICÍPIO</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>ESTADO</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>BANDEIRA</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>PRODUTO</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>UNIDADE DE MEDIDA</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>PREÇO DE REVENDA</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>DATA DA COLETA</t>
+          <t>PERÍODO: 27/09/2026 A 03/10/2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>11.111.111/0001-01</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>AUTO POSTO UM LTDA</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>POSTO UM</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>RUA A</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>CENTRO</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>01000-000</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>SÃO PAULO</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>SAO PAULO</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>BRANCA</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>GASOLINA COMUM</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>R$ / litro</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
-        <v>6.29</v>
-      </c>
-      <c r="O6" s="1" t="n">
-        <v>46294</v>
+          <t>COMBUSTÍVEL: TODOS</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>11.111.111/0001-01</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>AUTO POSTO UM LTDA</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>POSTO UM</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>RUA A</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>CENTRO</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>01000-000</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>SÃO PAULO</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>SAO PAULO</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>BRANCA</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>ETANOL HIDRATADO</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>R$ / litro</t>
-        </is>
-      </c>
-      <c r="N7" t="n">
-        <v>4.19</v>
-      </c>
-      <c r="O7" s="1" t="n">
-        <v>46294</v>
+          <t>TIPO RELATÓRIO: MUNICÍPIO</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>11.111.111/0001-01</t>
+          <t>CNPJ</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AUTO POSTO UM LTDA</t>
+          <t>RAZÃO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>POSTO UM</t>
+          <t>FANTASIA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>RUA A</t>
+          <t>ENDEREÇO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>NÚMERO</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>COMPLEMENTO</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>CENTRO</t>
+          <t>BAIRRO</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>01000-000</t>
+          <t>CEP</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>SÃO PAULO</t>
+          <t>MUNICÍPIO</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>SAO PAULO</t>
+          <t>ESTADO</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>BANDEIRA</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>OLEO DIESEL S10</t>
+          <t>PRODUTO</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>R$ / litro</t>
-        </is>
-      </c>
-      <c r="N8" t="n">
-        <v>6.09</v>
-      </c>
-      <c r="O8" s="1" t="n">
-        <v>46294</v>
+          <t>UNIDADE DE MEDIDA</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>PREÇO DE REVENDA</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>DATA DA COLETA</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>22.222.222/0001-02</t>
+          <t>11111111000101</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>POSTO DOIS LTDA</t>
+          <t>AUTO POSTO UM LTDA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DOIS</t>
+          <t>POSTO UM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AV B</t>
+          <t>RUA A</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>LOJA 1</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SÉ</t>
+          <t>CENTRO</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>01001-000</t>
+          <t>01000-000</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -779,12 +596,12 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>IPIRANGA</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>GASOLINA ADITIVADA</t>
+          <t>GASOLINA COMUM</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -793,7 +610,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>6.489999999999999</v>
+        <v>6.29</v>
       </c>
       <c r="O9" s="1" t="n">
         <v>46294</v>
@@ -802,42 +619,38 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>22.222.222/0001-02</t>
+          <t>11111111000101</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>POSTO DOIS LTDA</t>
+          <t>AUTO POSTO UM LTDA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DOIS</t>
+          <t>POSTO UM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>AV B</t>
+          <t>RUA A</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>LOJA 1</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SÉ</t>
+          <t>CENTRO</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>01001-000</t>
+          <t>01000-000</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -852,12 +665,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>IPIRANGA</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>OLEO DIESEL</t>
+          <t>ETANOL</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -866,7 +679,7 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>5.99</v>
+        <v>4.19</v>
       </c>
       <c r="O10" s="1" t="n">
         <v>46294</v>
@@ -875,42 +688,38 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>22.222.222/0001-02</t>
+          <t>11111111000101</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>POSTO DOIS LTDA</t>
+          <t>AUTO POSTO UM LTDA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DOIS</t>
+          <t>POSTO UM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>AV B</t>
+          <t>RUA A</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>LOJA 1</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>SÉ</t>
+          <t>CENTRO</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>01001-000</t>
+          <t>01000-000</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -925,21 +734,21 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>IPIRANGA</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>GNV</t>
+          <t>DIESEL S10</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>R$ / m³</t>
+          <t>R$ / litro</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>4.99</v>
+        <v>6.09</v>
       </c>
       <c r="O11" s="1" t="n">
         <v>46294</v>
@@ -948,344 +757,561 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>33.333.333/0001-03</t>
+          <t>22222222000102</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>REVENDA DE GAS TRES LTDA</t>
+          <t>POSTO DOIS LTDA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GAS TRES</t>
+          <t>DOIS</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>RUA C</t>
+          <t>AV B</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>LOJA 1</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>BOA VISTA</t>
+          <t>SÉ</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>50000-000</t>
+          <t>01001-000</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>RECIFE</t>
+          <t>SÃO PAULO</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>PERNAMBUCO</t>
+          <t>SAO PAULO</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>NACIONAL GAS</t>
+          <t>IPIRANGA</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GASOLINA ADITIVADA</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>R$ / 13 kg</t>
+          <t>R$ / litro</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>115</v>
+        <v>6.489999999999999</v>
       </c>
       <c r="O12" s="1" t="n">
-        <v>46295</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>44.444.444/0001-04</t>
+          <t>22222222000102</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>REVENDA QUATRO</t>
+          <t>POSTO DOIS LTDA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>QUATRO</t>
+          <t>DOIS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>RUA D</t>
+          <t>AV B</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>LOJA 1</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>BOA VIAGEM</t>
+          <t>SÉ</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>51000-000</t>
+          <t>01001-000</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>RECIFE</t>
+          <t>SÃO PAULO</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>SAO PAULO</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>ULTRAGAZ</t>
+          <t>IPIRANGA</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>DIESEL S500</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>R$ / 13 kg</t>
+          <t>R$ / litro</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>119.9</v>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
+        <v>5.99</v>
+      </c>
+      <c r="O13" s="1" t="n">
+        <v>46294</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>55.555.555/0001-05</t>
+          <t>22222222000102</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>REVENDA CINCO</t>
+          <t>POSTO DOIS LTDA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CINCO</t>
+          <t>DOIS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>RUA E</t>
+          <t>AV B</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>LOJA 1</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>CENTRO</t>
+          <t>SÉ</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>51000-000</t>
+          <t>01001-000</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>RECIFE</t>
+          <t>SÃO PAULO</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>PERNAMBUCO</t>
+          <t>SAO PAULO</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>IPIRANGA</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>GLP</t>
+          <t>GNV</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>R$ / 45 kg</t>
+          <t>R$ / m³</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>420</v>
+        <v>4.99</v>
       </c>
       <c r="O14" s="1" t="n">
-        <v>46295</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>66.666.666/0001-06</t>
+          <t>33333333000103</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>POSTO SEIS</t>
+          <t>REVENDA DE GAS TRES LTDA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SEIS</t>
+          <t>GAS TRES</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>RUA F</t>
+          <t>RUA C</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>CENTRO</t>
+          <t>BOA VISTA</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>20000-000</t>
+          <t>50000-000</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>NITERÓI</t>
+          <t>RECIFE</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>RIO DE JANEIRO</t>
+          <t>PERNAMBUCO</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>SHELL</t>
+          <t>NACIONAL GAS</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>GASOLINA COMUM</t>
+          <t>GLP</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>R$ / litro</t>
-        </is>
+          <t>R$ / 13 kg</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>115</v>
       </c>
       <c r="O15" s="1" t="n">
         <v>46295</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>77.777.777/0001-07</t>
-        </is>
+      <c r="A16" t="n">
+        <v>4444444000104</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>POSTO SETE</t>
+          <t>REVENDA QUATRO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SETE</t>
+          <t>QUATRO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>RUA G</t>
+          <t>RUA D</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
+          <t>BOA VIAGEM</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>51000-000</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>RECIFE</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ULTRAGAZ</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>GLP</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>R$ / 13 kg</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>119.9</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>55555555000105</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>REVENDA CINCO</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CINCO</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>RUA E</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
           <t>CENTRO</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>51000-000</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>RECIFE</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>PERNAMBUCO</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>BRANCA</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>GLP</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>R$ / 45 kg</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>420</v>
+      </c>
+      <c r="O17" s="1" t="n">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>66666666000106</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>POSTO SEIS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SEIS</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>RUA F</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>CENTRO</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>20000-000</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>NITERÓI</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>RIO DE JANEIRO</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>SHELL</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>GASOLINA COMUM</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>R$ / litro</t>
+        </is>
+      </c>
+      <c r="O18" s="1" t="n">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>77777777000107</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>POSTO SETE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>SETE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>RUA G</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>CENTRO</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>20000-000</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>NITERÓI</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>ESTADO INEXISTENTE</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>SHELL</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>GASOLINA COMUM</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>R$ / litro</t>
         </is>
       </c>
-      <c r="N16" t="n">
+      <c r="N19" t="n">
         <v>6.59</v>
       </c>
-      <c r="O16" s="1" t="n">
+      <c r="O19" s="1" t="n">
         <v>46295</v>
       </c>
     </row>

</xml_diff>